<commit_message>
ACTIVE INACTIVE IN VARIANT ON BASE OF EXCEL
</commit_message>
<xml_diff>
--- a/Full-LC-AUTO/data inputs/common/Price-Stock-Shipping-inputs.xlsx
+++ b/Full-LC-AUTO/data inputs/common/Price-Stock-Shipping-inputs.xlsx
@@ -397,34 +397,34 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:Z28"/>
+  <dimension ref="A1:Z29"/>
   <cols>
-    <col min="1" max="1" width="28.83203125" customWidth="1"/>
-    <col min="2" max="2" width="14.83203125" customWidth="1"/>
-    <col min="3" max="3" width="20.6640625" customWidth="1"/>
-    <col min="4" max="4" width="21.83203125" customWidth="1"/>
-    <col min="5" max="5" width="17.1640625" customWidth="1"/>
-    <col min="6" max="6" width="26.50390625" customWidth="1"/>
-    <col min="7" max="7" width="33.50390625" customWidth="1"/>
-    <col min="8" max="8" width="21.83203125" customWidth="1"/>
-    <col min="9" max="9" width="24.1640625" customWidth="1"/>
-    <col min="10" max="10" width="23.00390625" customWidth="1"/>
-    <col min="11" max="11" width="17.1640625" customWidth="1"/>
-    <col min="12" max="12" width="25.33203125" customWidth="1"/>
-    <col min="13" max="13" width="26.50390625" customWidth="1"/>
-    <col min="14" max="14" width="26.50390625" customWidth="1"/>
-    <col min="15" max="15" width="30.00390625" customWidth="1"/>
-    <col min="16" max="16" width="17.1640625" customWidth="1"/>
-    <col min="17" max="17" width="17.1640625" customWidth="1"/>
-    <col min="18" max="18" width="17.1640625" customWidth="1"/>
-    <col min="19" max="19" width="17.1640625" customWidth="1"/>
-    <col min="20" max="20" width="17.1640625" customWidth="1"/>
-    <col min="21" max="21" width="18.33203125" customWidth="1"/>
-    <col min="22" max="22" width="17.1640625" customWidth="1"/>
-    <col min="23" max="23" width="25.33203125" customWidth="1"/>
-    <col min="24" max="24" width="28.83203125" customWidth="1"/>
-    <col min="25" max="25" width="21.83203125" customWidth="1"/>
-    <col min="26" max="26" width="24.1640625" customWidth="1"/>
+    <col min="1" max="1" width="41.1640625" customWidth="1"/>
+    <col min="2" max="2" width="22.00390625" customWidth="1"/>
+    <col min="3" max="3" width="30.00390625" customWidth="1"/>
+    <col min="4" max="4" width="31.50390625" customWidth="1"/>
+    <col min="5" max="5" width="25.1640625" customWidth="1"/>
+    <col min="6" max="6" width="38.00390625" customWidth="1"/>
+    <col min="7" max="7" width="47.50390625" customWidth="1"/>
+    <col min="8" max="8" width="31.50390625" customWidth="1"/>
+    <col min="9" max="9" width="34.6640625" customWidth="1"/>
+    <col min="10" max="10" width="33.1640625" customWidth="1"/>
+    <col min="11" max="11" width="25.1640625" customWidth="1"/>
+    <col min="12" max="12" width="36.1640625" customWidth="1"/>
+    <col min="13" max="13" width="38.00390625" customWidth="1"/>
+    <col min="14" max="14" width="38.00390625" customWidth="1"/>
+    <col min="15" max="15" width="42.6640625" customWidth="1"/>
+    <col min="16" max="16" width="25.1640625" customWidth="1"/>
+    <col min="17" max="17" width="25.1640625" customWidth="1"/>
+    <col min="18" max="18" width="25.1640625" customWidth="1"/>
+    <col min="19" max="19" width="25.1640625" customWidth="1"/>
+    <col min="20" max="20" width="25.1640625" customWidth="1"/>
+    <col min="21" max="21" width="26.6640625" customWidth="1"/>
+    <col min="22" max="22" width="25.1640625" customWidth="1"/>
+    <col min="23" max="23" width="36.1640625" customWidth="1"/>
+    <col min="24" max="24" width="41.1640625" customWidth="1"/>
+    <col min="25" max="25" width="31.50390625" customWidth="1"/>
+    <col min="26" max="26" width="34.6640625" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -826,7 +826,7 @@
         <v>F-26-Beige-Baggy-Plain-Jeans-BEPJ-</v>
       </c>
       <c r="D6" t="str">
-        <v>Active</v>
+        <v>Inactive</v>
       </c>
       <c r="E6" t="str">
         <v>2499</v>
@@ -1359,13 +1359,13 @@
         <v>Trouser</v>
       </c>
       <c r="B13" t="str">
-        <v>M</v>
+        <v>26</v>
       </c>
       <c r="C13" t="str">
-        <v>F-M-TROUSER-BLACk-01-</v>
+        <v>F-XL-TROUSER-BLACk-01-</v>
       </c>
       <c r="D13" t="str">
-        <v>Active</v>
+        <v>Inactive</v>
       </c>
       <c r="E13" t="str">
         <v>2499</v>
@@ -1436,10 +1436,10 @@
         <v>Trouser</v>
       </c>
       <c r="B14" t="str">
-        <v>L</v>
+        <v>M</v>
       </c>
       <c r="C14" t="str">
-        <v>F-L-TROUSER-BLACk-01-</v>
+        <v>F-M-TROUSER-BLACk-01-</v>
       </c>
       <c r="D14" t="str">
         <v>Active</v>
@@ -1513,10 +1513,10 @@
         <v>Trouser</v>
       </c>
       <c r="B15" t="str">
-        <v>XL</v>
+        <v>L</v>
       </c>
       <c r="C15" t="str">
-        <v>F-XL-TROUSER-BLACk-01-</v>
+        <v>F-L-TROUSER-BLACk-01-</v>
       </c>
       <c r="D15" t="str">
         <v>Active</v>
@@ -1585,29 +1585,183 @@
         <v>Made In India</v>
       </c>
     </row>
-    <row r="25">
-      <c r="A25" t="str">
-        <v>How to use</v>
+    <row r="16">
+      <c r="A16" t="str">
+        <v>Trouser</v>
+      </c>
+      <c r="B16" t="str">
+        <v>XL</v>
+      </c>
+      <c r="C16" t="str">
+        <v>F-XL-TROUSER-BLACk-01-</v>
+      </c>
+      <c r="D16" t="str">
+        <v>Active</v>
+      </c>
+      <c r="E16" t="str">
+        <v>2499</v>
+      </c>
+      <c r="F16" t="str">
+        <v>359</v>
+      </c>
+      <c r="G16" t="str">
+        <v>1</v>
+      </c>
+      <c r="H16" t="str">
+        <v>Seller</v>
+      </c>
+      <c r="I16" t="str">
+        <v>express</v>
+      </c>
+      <c r="J16" t="str">
+        <v>1</v>
+      </c>
+      <c r="K16" t="str">
+        <v>250</v>
+      </c>
+      <c r="L16" t="str">
+        <v>Flipkart</v>
+      </c>
+      <c r="M16" t="str">
+        <v>0</v>
+      </c>
+      <c r="N16" t="str">
+        <v>0</v>
+      </c>
+      <c r="O16" t="str">
+        <v>0</v>
+      </c>
+      <c r="P16" t="str">
+        <v>35</v>
+      </c>
+      <c r="Q16" t="str">
+        <v>27</v>
+      </c>
+      <c r="R16" t="str">
+        <v>2</v>
+      </c>
+      <c r="S16" t="str">
+        <v>0.25</v>
+      </c>
+      <c r="T16" t="str">
+        <v>6109</v>
+      </c>
+      <c r="V16" t="str">
+        <v>GST_APPAREL</v>
+      </c>
+      <c r="W16" t="str">
+        <v>India</v>
+      </c>
+      <c r="X16" t="str">
+        <v>Made In India</v>
+      </c>
+      <c r="Y16" t="str">
+        <v>Made In India</v>
+      </c>
+      <c r="Z16" t="str">
+        <v>Made In India</v>
+      </c>
+    </row>
+    <row r="17">
+      <c r="A17" t="str">
+        <v>Trouser</v>
+      </c>
+      <c r="B17" t="str">
+        <v>S</v>
+      </c>
+      <c r="C17" t="str">
+        <v>F-S-TROUSER-BLACk-01-</v>
+      </c>
+      <c r="D17" t="str">
+        <v>Inactive</v>
+      </c>
+      <c r="E17" t="str">
+        <v>2499</v>
+      </c>
+      <c r="F17" t="str">
+        <v>359</v>
+      </c>
+      <c r="G17" t="str">
+        <v>1</v>
+      </c>
+      <c r="H17" t="str">
+        <v>Seller</v>
+      </c>
+      <c r="I17" t="str">
+        <v>express</v>
+      </c>
+      <c r="J17" t="str">
+        <v>1</v>
+      </c>
+      <c r="K17" t="str">
+        <v>250</v>
+      </c>
+      <c r="L17" t="str">
+        <v>Flipkart</v>
+      </c>
+      <c r="M17" t="str">
+        <v>0</v>
+      </c>
+      <c r="N17" t="str">
+        <v>0</v>
+      </c>
+      <c r="O17" t="str">
+        <v>0</v>
+      </c>
+      <c r="P17" t="str">
+        <v>35</v>
+      </c>
+      <c r="Q17" t="str">
+        <v>27</v>
+      </c>
+      <c r="R17" t="str">
+        <v>2</v>
+      </c>
+      <c r="S17" t="str">
+        <v>0.25</v>
+      </c>
+      <c r="T17" t="str">
+        <v>6109</v>
+      </c>
+      <c r="V17" t="str">
+        <v>GST_APPAREL</v>
+      </c>
+      <c r="W17" t="str">
+        <v>India</v>
+      </c>
+      <c r="X17" t="str">
+        <v>Made In India</v>
+      </c>
+      <c r="Y17" t="str">
+        <v>Made In India</v>
+      </c>
+      <c r="Z17" t="str">
+        <v>Made In India</v>
       </c>
     </row>
     <row r="26">
       <c r="A26" t="str">
-        <v>Use one row per product/size combination.</v>
+        <v>How to use</v>
       </c>
     </row>
     <row r="27">
       <c r="A27" t="str">
-        <v>The bot can generate a random 7-character suffix and append it to the Seller SKU ID value when filling the page.</v>
+        <v>Use one row per product/size combination.</v>
       </c>
     </row>
     <row r="28">
       <c r="A28" t="str">
+        <v>The bot can generate a random 7-character suffix and append it to the Seller SKU ID value when filling the page.</v>
+      </c>
+    </row>
+    <row r="29">
+      <c r="A29" t="str">
         <v>Do not rename headers.</v>
       </c>
     </row>
   </sheetData>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:Z28"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:Z29"/>
   </ignoredErrors>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
added TRACK PANT TO LC
</commit_message>
<xml_diff>
--- a/Full-LC-AUTO/data inputs/common/Price-Stock-Shipping-inputs.xlsx
+++ b/Full-LC-AUTO/data inputs/common/Price-Stock-Shipping-inputs.xlsx
@@ -11,7 +11,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="324" uniqueCount="70">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="371" uniqueCount="74">
   <si>
     <t>kind</t>
   </si>
@@ -97,7 +97,7 @@
     <t>BEIGE</t>
   </si>
   <si>
-    <t>F-34-Beige-Baggy-Plain-Jeans-BEPJ-</t>
+    <t>FB-34-Beige-Baggy-Plain-Jeans-BEPJ-</t>
   </si>
   <si>
     <t>Active</t>
@@ -121,16 +121,16 @@
     <t>Made In India</t>
   </si>
   <si>
-    <t>F-32-Beige-Baggy-Plain-Jeans-BEPJ-</t>
-  </si>
-  <si>
-    <t>F-30-Beige-Baggy-Plain-Jeans-BEPJ-</t>
-  </si>
-  <si>
-    <t>F-28-Beige-Baggy-Plain-Jeans-BEPJ-</t>
-  </si>
-  <si>
-    <t>F-26-Beige-Baggy-Plain-Jeans-BEPJ-</t>
+    <t>FB-32-Beige-Baggy-Plain-Jeans-BEPJ-</t>
+  </si>
+  <si>
+    <t>FB-30-Beige-Baggy-Plain-Jeans-BEPJ-</t>
+  </si>
+  <si>
+    <t>FB-28-Beige-Baggy-Plain-Jeans-BEPJ-</t>
+  </si>
+  <si>
+    <t>FB-26-Beige-Baggy-Plain-Jeans-BEPJ-</t>
   </si>
   <si>
     <t>Inactive</t>
@@ -139,19 +139,19 @@
     <t>ICE</t>
   </si>
   <si>
-    <t>F-34-ICE-Baggy-Plain-Jeans-BEPJ-</t>
-  </si>
-  <si>
-    <t>F-32-ICE-Baggy-Plain-Jeans-BEPJ-</t>
-  </si>
-  <si>
-    <t>F-30-ICE-Baggy-Plain-Jeans-BEPJ-</t>
-  </si>
-  <si>
-    <t>F-28-ICE-Baggy-Plain-Jeans-BEPJ-</t>
-  </si>
-  <si>
-    <t>F-26-ICE-Baggy-Plain-Jeans-BEPJ-</t>
+    <t>FB-34-ICE-Baggy-Plain-Jeans-BEPJ-</t>
+  </si>
+  <si>
+    <t>FB-32-ICE-Baggy-Plain-Jeans-BEPJ-</t>
+  </si>
+  <si>
+    <t>FB-30-ICE-Baggy-Plain-Jeans-BEPJ-</t>
+  </si>
+  <si>
+    <t>FB-28-ICE-Baggy-Plain-Jeans-BEPJ-</t>
+  </si>
+  <si>
+    <t>FB-26-ICE-Baggy-Plain-Jeans-BEPJ-</t>
   </si>
   <si>
     <t>Shorts</t>
@@ -160,34 +160,34 @@
     <t>XL</t>
   </si>
   <si>
-    <t>F-Shorts-XL-Black-01-</t>
+    <t>FB-Shorts-XL-Black-01-</t>
   </si>
   <si>
     <t>L</t>
   </si>
   <si>
-    <t>F-Shorts-L-Black-01-</t>
+    <t>FB-Shorts-L-Black-01-</t>
   </si>
   <si>
     <t>M</t>
   </si>
   <si>
-    <t>F-Shorts-M-Black-01-</t>
+    <t>FB-Shorts-M-Black-01-</t>
   </si>
   <si>
     <t>Trouser</t>
   </si>
   <si>
-    <t>F-M-TROUSER-BLACk-01-</t>
-  </si>
-  <si>
-    <t>F-L-TROUSER-BLACk-01-</t>
-  </si>
-  <si>
-    <t>F-XL-TROUSER-BLACk-01-</t>
-  </si>
-  <si>
-    <t>F-S-TROUSER-BLACk-01-</t>
+    <t>FB-M-TROUSER-BLACk-01-</t>
+  </si>
+  <si>
+    <t>FB-L-TROUSER-BLACk-01-</t>
+  </si>
+  <si>
+    <t>FB-XL-TROUSER-BLACk-01-</t>
+  </si>
+  <si>
+    <t>FB-S-TROUSER-BLACk-01-</t>
   </si>
   <si>
     <t>S</t>
@@ -196,22 +196,34 @@
     <t>Black-baggy</t>
   </si>
   <si>
-    <t>F-34-Black-Baggy-Plain-Jeans-BEPJ-</t>
-  </si>
-  <si>
-    <t>F-32-Black-Baggy-Plain-Jeans-BEPJ-</t>
-  </si>
-  <si>
-    <t>F-30-Black-Baggy-Plain-Jeans-BEPJ-</t>
-  </si>
-  <si>
-    <t>F-28-Black-Baggy-Plain-Jeans-BEPJ-</t>
-  </si>
-  <si>
-    <t>F-26-Black-Baggy-Plain-Jeans-BEPJ-</t>
-  </si>
-  <si>
-    <t>How to use</t>
+    <t>FB-34-Black-Baggy-Plain-Jeans-BEPJ-</t>
+  </si>
+  <si>
+    <t>FB-32-Black-Baggy-Plain-Jeans-BEPJ-</t>
+  </si>
+  <si>
+    <t>FB-30-Black-Baggy-Plain-Jeans-BEPJ-</t>
+  </si>
+  <si>
+    <t>FB-28-Black-Baggy-Plain-Jeans-BEPJ-</t>
+  </si>
+  <si>
+    <t>FB-26-Black-Baggy-Plain-Jeans-BEPJ-</t>
+  </si>
+  <si>
+    <t>Track Pant</t>
+  </si>
+  <si>
+    <t>FB-M-TRACK-PANT-BLACk-01-</t>
+  </si>
+  <si>
+    <t>FB-L-TRACK-PANT-BLACk-01-</t>
+  </si>
+  <si>
+    <t>FB-XL-TRACK-PANT-BLACk-01-</t>
+  </si>
+  <si>
+    <t>FB-S-TRACK-PANT-BLACk-01-</t>
   </si>
   <si>
     <t>Use one row per product/size combination.</t>
@@ -597,7 +609,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
-  <dimension ref="A1:AA34"/>
+  <dimension ref="A1:AA42"/>
   <sheetFormatPr defaultRowHeight="15" outlineLevelRow="0" outlineLevelCol="0" x14ac:dyDescent="55"/>
   <cols>
     <col min="1" max="1" width="42.142857142857146" customWidth="1"/>
@@ -716,7 +728,7 @@
         <v>29</v>
       </c>
       <c r="E2">
-        <v>2499</v>
+        <v>1499</v>
       </c>
       <c r="F2">
         <v>459</v>
@@ -796,7 +808,7 @@
         <v>29</v>
       </c>
       <c r="E3">
-        <v>2499</v>
+        <v>1499</v>
       </c>
       <c r="F3">
         <v>459</v>
@@ -876,7 +888,7 @@
         <v>29</v>
       </c>
       <c r="E4">
-        <v>2499</v>
+        <v>1499</v>
       </c>
       <c r="F4">
         <v>459</v>
@@ -956,7 +968,7 @@
         <v>29</v>
       </c>
       <c r="E5">
-        <v>2499</v>
+        <v>1499</v>
       </c>
       <c r="F5">
         <v>459</v>
@@ -1036,7 +1048,7 @@
         <v>40</v>
       </c>
       <c r="E6">
-        <v>2499</v>
+        <v>1499</v>
       </c>
       <c r="F6">
         <v>459</v>
@@ -1116,7 +1128,7 @@
         <v>29</v>
       </c>
       <c r="E7">
-        <v>2499</v>
+        <v>1499</v>
       </c>
       <c r="F7">
         <v>469</v>
@@ -1196,7 +1208,7 @@
         <v>29</v>
       </c>
       <c r="E8">
-        <v>2499</v>
+        <v>1499</v>
       </c>
       <c r="F8">
         <v>469</v>
@@ -1276,7 +1288,7 @@
         <v>29</v>
       </c>
       <c r="E9">
-        <v>2499</v>
+        <v>1499</v>
       </c>
       <c r="F9">
         <v>469</v>
@@ -1356,7 +1368,7 @@
         <v>29</v>
       </c>
       <c r="E10">
-        <v>2499</v>
+        <v>1499</v>
       </c>
       <c r="F10">
         <v>469</v>
@@ -1436,7 +1448,7 @@
         <v>40</v>
       </c>
       <c r="E11">
-        <v>2499</v>
+        <v>1499</v>
       </c>
       <c r="F11">
         <v>469</v>
@@ -2396,7 +2408,7 @@
         <v>29</v>
       </c>
       <c r="E23">
-        <v>2499</v>
+        <v>1499</v>
       </c>
       <c r="F23">
         <v>429</v>
@@ -2476,7 +2488,7 @@
         <v>29</v>
       </c>
       <c r="E24">
-        <v>2499</v>
+        <v>1499</v>
       </c>
       <c r="F24">
         <v>429</v>
@@ -2556,7 +2568,7 @@
         <v>29</v>
       </c>
       <c r="E25">
-        <v>2499</v>
+        <v>1499</v>
       </c>
       <c r="F25">
         <v>429</v>
@@ -2636,7 +2648,7 @@
         <v>29</v>
       </c>
       <c r="E26">
-        <v>2499</v>
+        <v>1499</v>
       </c>
       <c r="F26">
         <v>429</v>
@@ -2716,7 +2728,7 @@
         <v>40</v>
       </c>
       <c r="E27">
-        <v>2499</v>
+        <v>1499</v>
       </c>
       <c r="F27">
         <v>429</v>
@@ -2782,24 +2794,339 @@
         <v>35</v>
       </c>
     </row>
-    <row r="31" spans="1:1" x14ac:dyDescent="0.25">
+    <row r="28" spans="1:27" x14ac:dyDescent="0.25">
+      <c r="A28" t="s">
+        <v>66</v>
+      </c>
+      <c r="B28" t="s">
+        <v>52</v>
+      </c>
+      <c r="C28" t="s">
+        <v>67</v>
+      </c>
+      <c r="D28" t="s">
+        <v>29</v>
+      </c>
+      <c r="E28">
+        <v>999</v>
+      </c>
+      <c r="F28">
+        <v>315</v>
+      </c>
+      <c r="G28">
+        <v>279</v>
+      </c>
+      <c r="H28">
+        <v>1</v>
+      </c>
+      <c r="I28" t="s">
+        <v>30</v>
+      </c>
+      <c r="J28" t="s">
+        <v>31</v>
+      </c>
+      <c r="K28">
+        <v>1</v>
+      </c>
+      <c r="L28">
+        <v>250</v>
+      </c>
+      <c r="M28" t="s">
+        <v>32</v>
+      </c>
+      <c r="N28">
+        <v>0</v>
+      </c>
+      <c r="O28">
+        <v>0</v>
+      </c>
+      <c r="P28">
+        <v>0</v>
+      </c>
+      <c r="Q28">
+        <v>35</v>
+      </c>
+      <c r="R28">
+        <v>27</v>
+      </c>
+      <c r="S28">
+        <v>2</v>
+      </c>
+      <c r="T28">
+        <v>0.25</v>
+      </c>
+      <c r="U28">
+        <v>6109</v>
+      </c>
+      <c r="W28" t="s">
+        <v>33</v>
+      </c>
+      <c r="X28" t="s">
+        <v>34</v>
+      </c>
+      <c r="Y28" t="s">
+        <v>35</v>
+      </c>
+      <c r="Z28" t="s">
+        <v>35</v>
+      </c>
+      <c r="AA28" t="s">
+        <v>35</v>
+      </c>
+    </row>
+    <row r="29" spans="1:27" x14ac:dyDescent="0.25">
+      <c r="A29" t="s">
+        <v>66</v>
+      </c>
+      <c r="B29" t="s">
+        <v>50</v>
+      </c>
+      <c r="C29" t="s">
+        <v>68</v>
+      </c>
+      <c r="D29" t="s">
+        <v>29</v>
+      </c>
+      <c r="E29">
+        <v>999</v>
+      </c>
+      <c r="F29">
+        <v>315</v>
+      </c>
+      <c r="G29">
+        <v>279</v>
+      </c>
+      <c r="H29">
+        <v>1</v>
+      </c>
+      <c r="I29" t="s">
+        <v>30</v>
+      </c>
+      <c r="J29" t="s">
+        <v>31</v>
+      </c>
+      <c r="K29">
+        <v>1</v>
+      </c>
+      <c r="L29">
+        <v>250</v>
+      </c>
+      <c r="M29" t="s">
+        <v>32</v>
+      </c>
+      <c r="N29">
+        <v>0</v>
+      </c>
+      <c r="O29">
+        <v>0</v>
+      </c>
+      <c r="P29">
+        <v>0</v>
+      </c>
+      <c r="Q29">
+        <v>35</v>
+      </c>
+      <c r="R29">
+        <v>27</v>
+      </c>
+      <c r="S29">
+        <v>2</v>
+      </c>
+      <c r="T29">
+        <v>0.25</v>
+      </c>
+      <c r="U29">
+        <v>6109</v>
+      </c>
+      <c r="W29" t="s">
+        <v>33</v>
+      </c>
+      <c r="X29" t="s">
+        <v>34</v>
+      </c>
+      <c r="Y29" t="s">
+        <v>35</v>
+      </c>
+      <c r="Z29" t="s">
+        <v>35</v>
+      </c>
+      <c r="AA29" t="s">
+        <v>35</v>
+      </c>
+    </row>
+    <row r="30" spans="1:27" x14ac:dyDescent="0.25">
+      <c r="A30" t="s">
+        <v>66</v>
+      </c>
+      <c r="B30" t="s">
+        <v>48</v>
+      </c>
+      <c r="C30" t="s">
+        <v>69</v>
+      </c>
+      <c r="D30" t="s">
+        <v>29</v>
+      </c>
+      <c r="E30">
+        <v>999</v>
+      </c>
+      <c r="F30">
+        <v>315</v>
+      </c>
+      <c r="G30">
+        <v>279</v>
+      </c>
+      <c r="H30">
+        <v>1</v>
+      </c>
+      <c r="I30" t="s">
+        <v>30</v>
+      </c>
+      <c r="J30" t="s">
+        <v>31</v>
+      </c>
+      <c r="K30">
+        <v>1</v>
+      </c>
+      <c r="L30">
+        <v>250</v>
+      </c>
+      <c r="M30" t="s">
+        <v>32</v>
+      </c>
+      <c r="N30">
+        <v>0</v>
+      </c>
+      <c r="O30">
+        <v>0</v>
+      </c>
+      <c r="P30">
+        <v>0</v>
+      </c>
+      <c r="Q30">
+        <v>35</v>
+      </c>
+      <c r="R30">
+        <v>27</v>
+      </c>
+      <c r="S30">
+        <v>2</v>
+      </c>
+      <c r="T30">
+        <v>0.25</v>
+      </c>
+      <c r="U30">
+        <v>6109</v>
+      </c>
+      <c r="W30" t="s">
+        <v>33</v>
+      </c>
+      <c r="X30" t="s">
+        <v>34</v>
+      </c>
+      <c r="Y30" t="s">
+        <v>35</v>
+      </c>
+      <c r="Z30" t="s">
+        <v>35</v>
+      </c>
+      <c r="AA30" t="s">
+        <v>35</v>
+      </c>
+    </row>
+    <row r="31" spans="1:27" x14ac:dyDescent="0.25">
       <c r="A31" t="s">
         <v>66</v>
       </c>
-    </row>
-    <row r="32" spans="1:1" x14ac:dyDescent="0.25">
-      <c r="A32" t="s">
-        <v>67</v>
-      </c>
-    </row>
-    <row r="33" spans="1:1" x14ac:dyDescent="0.25">
-      <c r="A33" t="s">
-        <v>68</v>
-      </c>
-    </row>
-    <row r="34" spans="1:1" x14ac:dyDescent="0.25">
-      <c r="A34" t="s">
-        <v>69</v>
+      <c r="B31" t="s">
+        <v>59</v>
+      </c>
+      <c r="C31" t="s">
+        <v>70</v>
+      </c>
+      <c r="D31" t="s">
+        <v>40</v>
+      </c>
+      <c r="E31">
+        <v>999</v>
+      </c>
+      <c r="F31">
+        <v>315</v>
+      </c>
+      <c r="G31">
+        <v>279</v>
+      </c>
+      <c r="H31">
+        <v>1</v>
+      </c>
+      <c r="I31" t="s">
+        <v>30</v>
+      </c>
+      <c r="J31" t="s">
+        <v>31</v>
+      </c>
+      <c r="K31">
+        <v>1</v>
+      </c>
+      <c r="L31">
+        <v>250</v>
+      </c>
+      <c r="M31" t="s">
+        <v>32</v>
+      </c>
+      <c r="N31">
+        <v>0</v>
+      </c>
+      <c r="O31">
+        <v>0</v>
+      </c>
+      <c r="P31">
+        <v>0</v>
+      </c>
+      <c r="Q31">
+        <v>35</v>
+      </c>
+      <c r="R31">
+        <v>27</v>
+      </c>
+      <c r="S31">
+        <v>2</v>
+      </c>
+      <c r="T31">
+        <v>0.25</v>
+      </c>
+      <c r="U31">
+        <v>6109</v>
+      </c>
+      <c r="W31" t="s">
+        <v>33</v>
+      </c>
+      <c r="X31" t="s">
+        <v>34</v>
+      </c>
+      <c r="Y31" t="s">
+        <v>35</v>
+      </c>
+      <c r="Z31" t="s">
+        <v>35</v>
+      </c>
+      <c r="AA31" t="s">
+        <v>35</v>
+      </c>
+    </row>
+    <row r="40" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A40" t="s">
+        <v>71</v>
+      </c>
+    </row>
+    <row r="41" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A41" t="s">
+        <v>72</v>
+      </c>
+    </row>
+    <row r="42" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A42" t="s">
+        <v>73</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
hid licence deeper, fixed start_batch no winfo error
</commit_message>
<xml_diff>
--- a/Full-LC-AUTO/data inputs/common/Price-Stock-Shipping-inputs.xlsx
+++ b/Full-LC-AUTO/data inputs/common/Price-Stock-Shipping-inputs.xlsx
@@ -133,25 +133,25 @@
     <t>FB-26-Beige-Baggy-Plain-Jeans-BEPJ-</t>
   </si>
   <si>
+    <t>ICE</t>
+  </si>
+  <si>
+    <t>FB-34-ICE-Baggy-Plain-Jeans-BEPJ-</t>
+  </si>
+  <si>
+    <t>FB-32-ICE-Baggy-Plain-Jeans-BEPJ-</t>
+  </si>
+  <si>
+    <t>FB-30-ICE-Baggy-Plain-Jeans-BEPJ-</t>
+  </si>
+  <si>
+    <t>FB-28-ICE-Baggy-Plain-Jeans-BEPJ-</t>
+  </si>
+  <si>
+    <t>FB-26-ICE-Baggy-Plain-Jeans-BEPJ-</t>
+  </si>
+  <si>
     <t>Inactive</t>
-  </si>
-  <si>
-    <t>ICE</t>
-  </si>
-  <si>
-    <t>FB-34-ICE-Baggy-Plain-Jeans-BEPJ-</t>
-  </si>
-  <si>
-    <t>FB-32-ICE-Baggy-Plain-Jeans-BEPJ-</t>
-  </si>
-  <si>
-    <t>FB-30-ICE-Baggy-Plain-Jeans-BEPJ-</t>
-  </si>
-  <si>
-    <t>FB-28-ICE-Baggy-Plain-Jeans-BEPJ-</t>
-  </si>
-  <si>
-    <t>FB-26-ICE-Baggy-Plain-Jeans-BEPJ-</t>
   </si>
   <si>
     <t>Shorts</t>
@@ -1045,7 +1045,7 @@
         <v>39</v>
       </c>
       <c r="D6" t="s">
-        <v>40</v>
+        <v>29</v>
       </c>
       <c r="E6">
         <v>1499</v>
@@ -1116,13 +1116,13 @@
     </row>
     <row r="7" spans="1:27" x14ac:dyDescent="0.25">
       <c r="A7" t="s">
+        <v>40</v>
+      </c>
+      <c r="B7">
+        <v>34</v>
+      </c>
+      <c r="C7" t="s">
         <v>41</v>
-      </c>
-      <c r="B7">
-        <v>34</v>
-      </c>
-      <c r="C7" t="s">
-        <v>42</v>
       </c>
       <c r="D7" t="s">
         <v>29</v>
@@ -1196,13 +1196,13 @@
     </row>
     <row r="8" spans="1:27" x14ac:dyDescent="0.25">
       <c r="A8" t="s">
-        <v>41</v>
+        <v>40</v>
       </c>
       <c r="B8">
         <v>32</v>
       </c>
       <c r="C8" t="s">
-        <v>43</v>
+        <v>42</v>
       </c>
       <c r="D8" t="s">
         <v>29</v>
@@ -1276,13 +1276,13 @@
     </row>
     <row r="9" spans="1:27" x14ac:dyDescent="0.25">
       <c r="A9" t="s">
-        <v>41</v>
+        <v>40</v>
       </c>
       <c r="B9">
         <v>30</v>
       </c>
       <c r="C9" t="s">
-        <v>44</v>
+        <v>43</v>
       </c>
       <c r="D9" t="s">
         <v>29</v>
@@ -1356,13 +1356,13 @@
     </row>
     <row r="10" spans="1:27" x14ac:dyDescent="0.25">
       <c r="A10" t="s">
-        <v>41</v>
+        <v>40</v>
       </c>
       <c r="B10">
         <v>28</v>
       </c>
       <c r="C10" t="s">
-        <v>45</v>
+        <v>44</v>
       </c>
       <c r="D10" t="s">
         <v>29</v>
@@ -1436,16 +1436,16 @@
     </row>
     <row r="11" spans="1:27" x14ac:dyDescent="0.25">
       <c r="A11" t="s">
-        <v>41</v>
+        <v>40</v>
       </c>
       <c r="B11">
         <v>26</v>
       </c>
       <c r="C11" t="s">
+        <v>45</v>
+      </c>
+      <c r="D11" t="s">
         <v>46</v>
-      </c>
-      <c r="D11" t="s">
-        <v>40</v>
       </c>
       <c r="E11">
         <v>1499</v>
@@ -2005,7 +2005,7 @@
         <v>58</v>
       </c>
       <c r="D18" t="s">
-        <v>40</v>
+        <v>46</v>
       </c>
       <c r="E18">
         <v>999</v>
@@ -2325,7 +2325,7 @@
         <v>58</v>
       </c>
       <c r="D22" t="s">
-        <v>40</v>
+        <v>46</v>
       </c>
       <c r="E22">
         <v>999</v>
@@ -2725,7 +2725,7 @@
         <v>65</v>
       </c>
       <c r="D27" t="s">
-        <v>40</v>
+        <v>29</v>
       </c>
       <c r="E27">
         <v>1499</v>
@@ -3045,7 +3045,7 @@
         <v>70</v>
       </c>
       <c r="D31" t="s">
-        <v>40</v>
+        <v>46</v>
       </c>
       <c r="E31">
         <v>999</v>

</xml_diff>

<commit_message>
data inputs for white baggy
</commit_message>
<xml_diff>
--- a/Full-LC-AUTO/data inputs/common/Price-Stock-Shipping-inputs.xlsx
+++ b/Full-LC-AUTO/data inputs/common/Price-Stock-Shipping-inputs.xlsx
@@ -1,17 +1,21 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" mc:Ignorable="x15">
-  <fileVersion appName="xl" lastEdited="5" lowestEdited="5" rupBuild="9303"/>
-  <workbookPr defaultThemeVersion="164011" filterPrivacy="1"/>
+<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="5" rupBuild="30131"/>
+  <workbookPr filterPrivacy="1"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{48F5E4CA-D0C9-4E99-ABF4-C7A03FF330E7}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <bookViews>
+    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="13176" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+  </bookViews>
   <sheets>
-    <sheet sheetId="1" name="Product Inputs" state="visible" r:id="rId4"/>
+    <sheet name="Product Inputs" sheetId="1" r:id="rId1"/>
   </sheets>
   <calcPr calcId="171027"/>
 </workbook>
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="371" uniqueCount="74">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="426" uniqueCount="80">
   <si>
     <t>kind</t>
   </si>
@@ -233,19 +237,37 @@
   </si>
   <si>
     <t>Do not rename headers.</t>
+  </si>
+  <si>
+    <t>FB-34-WHITE-Baggy-Plain-Jeans-BEPJ-</t>
+  </si>
+  <si>
+    <t>FB-32-WHITE-Baggy-Plain-Jeans-BEPJ-</t>
+  </si>
+  <si>
+    <t>FB-30-WHITE-Baggy-Plain-Jeans-BEPJ-</t>
+  </si>
+  <si>
+    <t>FB-28-WHITE-Baggy-Plain-Jeans-BEPJ-</t>
+  </si>
+  <si>
+    <t>FB-26-WHITE-Baggy-Plain-Jeans-BEPJ-</t>
+  </si>
+  <si>
+    <t>White-Baggy</t>
   </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
-<styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" mc:Ignorable="x14ac x16r2">
+<styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
   <fonts count="1" x14ac:knownFonts="1">
     <font>
+      <sz val="11"/>
       <color theme="1"/>
+      <name val="Calibri"/>
       <family val="2"/>
       <scheme val="minor"/>
-      <sz val="11"/>
-      <name val="Calibri"/>
     </font>
   </fonts>
   <fills count="2">
@@ -608,30 +630,30 @@
 </file>
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
   <dimension ref="A1:AA42"/>
-  <sheetFormatPr defaultRowHeight="15" outlineLevelRow="0" outlineLevelCol="0" x14ac:dyDescent="55"/>
+  <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
-    <col min="1" max="1" width="42.142857142857146" customWidth="1"/>
-    <col min="2" max="2" width="26.571428571428573" customWidth="1"/>
-    <col min="3" max="3" width="35.857142857142854" customWidth="1"/>
-    <col min="4" max="4" width="37.714285714285715" customWidth="1"/>
-    <col min="5" max="6" width="30.142857142857142" customWidth="1"/>
-    <col min="7" max="8" width="42.142857142857146" customWidth="1"/>
-    <col min="9" max="9" width="37.714285714285715" customWidth="1"/>
-    <col min="10" max="10" width="41.142857142857146" customWidth="1"/>
-    <col min="11" max="11" width="39.57142857142857" customWidth="1"/>
-    <col min="12" max="12" width="30.142857142857142" customWidth="1"/>
-    <col min="13" max="16" width="42.142857142857146" customWidth="1"/>
-    <col min="17" max="21" width="30.142857142857142" customWidth="1"/>
-    <col min="22" max="22" width="31.857142857142858" customWidth="1"/>
-    <col min="23" max="23" width="30.142857142857142" customWidth="1"/>
-    <col min="24" max="25" width="42.142857142857146" customWidth="1"/>
-    <col min="26" max="26" width="37.714285714285715" customWidth="1"/>
-    <col min="27" max="27" width="41.142857142857146" customWidth="1"/>
+    <col min="1" max="1" width="42.109375" customWidth="1"/>
+    <col min="2" max="2" width="26.5546875" customWidth="1"/>
+    <col min="3" max="3" width="35.88671875" customWidth="1"/>
+    <col min="4" max="4" width="37.6640625" customWidth="1"/>
+    <col min="5" max="6" width="30.109375" customWidth="1"/>
+    <col min="7" max="8" width="42.109375" customWidth="1"/>
+    <col min="9" max="9" width="37.6640625" customWidth="1"/>
+    <col min="10" max="10" width="41.109375" customWidth="1"/>
+    <col min="11" max="11" width="39.5546875" customWidth="1"/>
+    <col min="12" max="12" width="30.109375" customWidth="1"/>
+    <col min="13" max="16" width="42.109375" customWidth="1"/>
+    <col min="17" max="21" width="30.109375" customWidth="1"/>
+    <col min="22" max="22" width="31.88671875" customWidth="1"/>
+    <col min="23" max="23" width="30.109375" customWidth="1"/>
+    <col min="24" max="25" width="42.109375" customWidth="1"/>
+    <col min="26" max="26" width="37.6640625" customWidth="1"/>
+    <col min="27" max="27" width="41.109375" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:27" x14ac:dyDescent="0.25">
+    <row r="1" spans="1:27" x14ac:dyDescent="0.3">
       <c r="A1" t="s">
         <v>0</v>
       </c>
@@ -714,7 +736,7 @@
         <v>26</v>
       </c>
     </row>
-    <row r="2" spans="1:27" x14ac:dyDescent="0.25">
+    <row r="2" spans="1:27" x14ac:dyDescent="0.3">
       <c r="A2" t="s">
         <v>27</v>
       </c>
@@ -773,7 +795,7 @@
         <v>2</v>
       </c>
       <c r="T2">
-        <v>0.465</v>
+        <v>0.46500000000000002</v>
       </c>
       <c r="U2">
         <v>62034200</v>
@@ -794,7 +816,7 @@
         <v>35</v>
       </c>
     </row>
-    <row r="3" spans="1:27" x14ac:dyDescent="0.25">
+    <row r="3" spans="1:27" x14ac:dyDescent="0.3">
       <c r="A3" t="s">
         <v>27</v>
       </c>
@@ -853,7 +875,7 @@
         <v>2</v>
       </c>
       <c r="T3">
-        <v>0.465</v>
+        <v>0.46500000000000002</v>
       </c>
       <c r="U3">
         <v>62034200</v>
@@ -874,7 +896,7 @@
         <v>35</v>
       </c>
     </row>
-    <row r="4" spans="1:27" x14ac:dyDescent="0.25">
+    <row r="4" spans="1:27" x14ac:dyDescent="0.3">
       <c r="A4" t="s">
         <v>27</v>
       </c>
@@ -933,7 +955,7 @@
         <v>2</v>
       </c>
       <c r="T4">
-        <v>0.465</v>
+        <v>0.46500000000000002</v>
       </c>
       <c r="U4">
         <v>62034200</v>
@@ -954,7 +976,7 @@
         <v>35</v>
       </c>
     </row>
-    <row r="5" spans="1:27" x14ac:dyDescent="0.25">
+    <row r="5" spans="1:27" x14ac:dyDescent="0.3">
       <c r="A5" t="s">
         <v>27</v>
       </c>
@@ -1013,7 +1035,7 @@
         <v>2</v>
       </c>
       <c r="T5">
-        <v>0.465</v>
+        <v>0.46500000000000002</v>
       </c>
       <c r="U5">
         <v>62034200</v>
@@ -1034,7 +1056,7 @@
         <v>35</v>
       </c>
     </row>
-    <row r="6" spans="1:27" x14ac:dyDescent="0.25">
+    <row r="6" spans="1:27" x14ac:dyDescent="0.3">
       <c r="A6" t="s">
         <v>27</v>
       </c>
@@ -1093,7 +1115,7 @@
         <v>2</v>
       </c>
       <c r="T6">
-        <v>0.465</v>
+        <v>0.46500000000000002</v>
       </c>
       <c r="U6">
         <v>62034200</v>
@@ -1114,7 +1136,7 @@
         <v>35</v>
       </c>
     </row>
-    <row r="7" spans="1:27" x14ac:dyDescent="0.25">
+    <row r="7" spans="1:27" x14ac:dyDescent="0.3">
       <c r="A7" t="s">
         <v>40</v>
       </c>
@@ -1173,7 +1195,7 @@
         <v>2</v>
       </c>
       <c r="T7">
-        <v>0.465</v>
+        <v>0.46500000000000002</v>
       </c>
       <c r="U7">
         <v>62034200</v>
@@ -1194,7 +1216,7 @@
         <v>35</v>
       </c>
     </row>
-    <row r="8" spans="1:27" x14ac:dyDescent="0.25">
+    <row r="8" spans="1:27" x14ac:dyDescent="0.3">
       <c r="A8" t="s">
         <v>40</v>
       </c>
@@ -1253,7 +1275,7 @@
         <v>2</v>
       </c>
       <c r="T8">
-        <v>0.465</v>
+        <v>0.46500000000000002</v>
       </c>
       <c r="U8">
         <v>62034200</v>
@@ -1274,7 +1296,7 @@
         <v>35</v>
       </c>
     </row>
-    <row r="9" spans="1:27" x14ac:dyDescent="0.25">
+    <row r="9" spans="1:27" x14ac:dyDescent="0.3">
       <c r="A9" t="s">
         <v>40</v>
       </c>
@@ -1333,7 +1355,7 @@
         <v>2</v>
       </c>
       <c r="T9">
-        <v>0.465</v>
+        <v>0.46500000000000002</v>
       </c>
       <c r="U9">
         <v>62034200</v>
@@ -1354,7 +1376,7 @@
         <v>35</v>
       </c>
     </row>
-    <row r="10" spans="1:27" x14ac:dyDescent="0.25">
+    <row r="10" spans="1:27" x14ac:dyDescent="0.3">
       <c r="A10" t="s">
         <v>40</v>
       </c>
@@ -1413,7 +1435,7 @@
         <v>2</v>
       </c>
       <c r="T10">
-        <v>0.465</v>
+        <v>0.46500000000000002</v>
       </c>
       <c r="U10">
         <v>62034200</v>
@@ -1434,7 +1456,7 @@
         <v>35</v>
       </c>
     </row>
-    <row r="11" spans="1:27" x14ac:dyDescent="0.25">
+    <row r="11" spans="1:27" x14ac:dyDescent="0.3">
       <c r="A11" t="s">
         <v>40</v>
       </c>
@@ -1493,7 +1515,7 @@
         <v>2</v>
       </c>
       <c r="T11">
-        <v>0.465</v>
+        <v>0.46500000000000002</v>
       </c>
       <c r="U11">
         <v>62034200</v>
@@ -1514,7 +1536,7 @@
         <v>35</v>
       </c>
     </row>
-    <row r="12" spans="1:27" x14ac:dyDescent="0.25">
+    <row r="12" spans="1:27" x14ac:dyDescent="0.3">
       <c r="A12" t="s">
         <v>47</v>
       </c>
@@ -1594,7 +1616,7 @@
         <v>35</v>
       </c>
     </row>
-    <row r="13" spans="1:27" x14ac:dyDescent="0.25">
+    <row r="13" spans="1:27" x14ac:dyDescent="0.3">
       <c r="A13" t="s">
         <v>47</v>
       </c>
@@ -1674,7 +1696,7 @@
         <v>35</v>
       </c>
     </row>
-    <row r="14" spans="1:27" x14ac:dyDescent="0.25">
+    <row r="14" spans="1:27" x14ac:dyDescent="0.3">
       <c r="A14" t="s">
         <v>47</v>
       </c>
@@ -1754,7 +1776,7 @@
         <v>35</v>
       </c>
     </row>
-    <row r="15" spans="1:27" x14ac:dyDescent="0.25">
+    <row r="15" spans="1:27" x14ac:dyDescent="0.3">
       <c r="A15" t="s">
         <v>54</v>
       </c>
@@ -1834,7 +1856,7 @@
         <v>35</v>
       </c>
     </row>
-    <row r="16" spans="1:27" x14ac:dyDescent="0.25">
+    <row r="16" spans="1:27" x14ac:dyDescent="0.3">
       <c r="A16" t="s">
         <v>54</v>
       </c>
@@ -1914,7 +1936,7 @@
         <v>35</v>
       </c>
     </row>
-    <row r="17" spans="1:27" x14ac:dyDescent="0.25">
+    <row r="17" spans="1:27" x14ac:dyDescent="0.3">
       <c r="A17" t="s">
         <v>54</v>
       </c>
@@ -1994,7 +2016,7 @@
         <v>35</v>
       </c>
     </row>
-    <row r="18" spans="1:27" x14ac:dyDescent="0.25">
+    <row r="18" spans="1:27" x14ac:dyDescent="0.3">
       <c r="A18" t="s">
         <v>54</v>
       </c>
@@ -2074,7 +2096,7 @@
         <v>35</v>
       </c>
     </row>
-    <row r="19" spans="1:27" x14ac:dyDescent="0.25">
+    <row r="19" spans="1:27" x14ac:dyDescent="0.3">
       <c r="A19" t="s">
         <v>54</v>
       </c>
@@ -2154,7 +2176,7 @@
         <v>35</v>
       </c>
     </row>
-    <row r="20" spans="1:27" x14ac:dyDescent="0.25">
+    <row r="20" spans="1:27" x14ac:dyDescent="0.3">
       <c r="A20" t="s">
         <v>54</v>
       </c>
@@ -2234,7 +2256,7 @@
         <v>35</v>
       </c>
     </row>
-    <row r="21" spans="1:27" x14ac:dyDescent="0.25">
+    <row r="21" spans="1:27" x14ac:dyDescent="0.3">
       <c r="A21" t="s">
         <v>54</v>
       </c>
@@ -2314,7 +2336,7 @@
         <v>35</v>
       </c>
     </row>
-    <row r="22" spans="1:27" x14ac:dyDescent="0.25">
+    <row r="22" spans="1:27" x14ac:dyDescent="0.3">
       <c r="A22" t="s">
         <v>54</v>
       </c>
@@ -2394,7 +2416,7 @@
         <v>35</v>
       </c>
     </row>
-    <row r="23" spans="1:27" x14ac:dyDescent="0.25">
+    <row r="23" spans="1:27" x14ac:dyDescent="0.3">
       <c r="A23" t="s">
         <v>60</v>
       </c>
@@ -2453,7 +2475,7 @@
         <v>2</v>
       </c>
       <c r="T23">
-        <v>0.465</v>
+        <v>0.46500000000000002</v>
       </c>
       <c r="U23">
         <v>62034200</v>
@@ -2474,7 +2496,7 @@
         <v>35</v>
       </c>
     </row>
-    <row r="24" spans="1:27" x14ac:dyDescent="0.25">
+    <row r="24" spans="1:27" x14ac:dyDescent="0.3">
       <c r="A24" t="s">
         <v>60</v>
       </c>
@@ -2533,7 +2555,7 @@
         <v>2</v>
       </c>
       <c r="T24">
-        <v>0.465</v>
+        <v>0.46500000000000002</v>
       </c>
       <c r="U24">
         <v>62034200</v>
@@ -2554,7 +2576,7 @@
         <v>35</v>
       </c>
     </row>
-    <row r="25" spans="1:27" x14ac:dyDescent="0.25">
+    <row r="25" spans="1:27" x14ac:dyDescent="0.3">
       <c r="A25" t="s">
         <v>60</v>
       </c>
@@ -2613,7 +2635,7 @@
         <v>2</v>
       </c>
       <c r="T25">
-        <v>0.465</v>
+        <v>0.46500000000000002</v>
       </c>
       <c r="U25">
         <v>62034200</v>
@@ -2634,7 +2656,7 @@
         <v>35</v>
       </c>
     </row>
-    <row r="26" spans="1:27" x14ac:dyDescent="0.25">
+    <row r="26" spans="1:27" x14ac:dyDescent="0.3">
       <c r="A26" t="s">
         <v>60</v>
       </c>
@@ -2693,7 +2715,7 @@
         <v>2</v>
       </c>
       <c r="T26">
-        <v>0.465</v>
+        <v>0.46500000000000002</v>
       </c>
       <c r="U26">
         <v>62034200</v>
@@ -2714,7 +2736,7 @@
         <v>35</v>
       </c>
     </row>
-    <row r="27" spans="1:27" x14ac:dyDescent="0.25">
+    <row r="27" spans="1:27" x14ac:dyDescent="0.3">
       <c r="A27" t="s">
         <v>60</v>
       </c>
@@ -2773,7 +2795,7 @@
         <v>2</v>
       </c>
       <c r="T27">
-        <v>0.465</v>
+        <v>0.46500000000000002</v>
       </c>
       <c r="U27">
         <v>62034200</v>
@@ -2794,7 +2816,7 @@
         <v>35</v>
       </c>
     </row>
-    <row r="28" spans="1:27" x14ac:dyDescent="0.25">
+    <row r="28" spans="1:27" x14ac:dyDescent="0.3">
       <c r="A28" t="s">
         <v>66</v>
       </c>
@@ -2874,7 +2896,7 @@
         <v>35</v>
       </c>
     </row>
-    <row r="29" spans="1:27" x14ac:dyDescent="0.25">
+    <row r="29" spans="1:27" x14ac:dyDescent="0.3">
       <c r="A29" t="s">
         <v>66</v>
       </c>
@@ -2954,7 +2976,7 @@
         <v>35</v>
       </c>
     </row>
-    <row r="30" spans="1:27" x14ac:dyDescent="0.25">
+    <row r="30" spans="1:27" x14ac:dyDescent="0.3">
       <c r="A30" t="s">
         <v>66</v>
       </c>
@@ -3034,7 +3056,7 @@
         <v>35</v>
       </c>
     </row>
-    <row r="31" spans="1:27" x14ac:dyDescent="0.25">
+    <row r="31" spans="1:27" x14ac:dyDescent="0.3">
       <c r="A31" t="s">
         <v>66</v>
       </c>
@@ -3114,23 +3136,423 @@
         <v>35</v>
       </c>
     </row>
-    <row r="40" spans="1:1" x14ac:dyDescent="0.25">
+    <row r="32" spans="1:27" x14ac:dyDescent="0.3">
+      <c r="A32" t="s">
+        <v>79</v>
+      </c>
+      <c r="B32">
+        <v>34</v>
+      </c>
+      <c r="C32" t="s">
+        <v>74</v>
+      </c>
+      <c r="D32" t="s">
+        <v>29</v>
+      </c>
+      <c r="E32">
+        <v>1499</v>
+      </c>
+      <c r="F32">
+        <v>459</v>
+      </c>
+      <c r="G32">
+        <v>442</v>
+      </c>
+      <c r="H32">
+        <v>1</v>
+      </c>
+      <c r="I32" t="s">
+        <v>30</v>
+      </c>
+      <c r="J32" t="s">
+        <v>31</v>
+      </c>
+      <c r="K32">
+        <v>1</v>
+      </c>
+      <c r="L32">
+        <v>250</v>
+      </c>
+      <c r="M32" t="s">
+        <v>32</v>
+      </c>
+      <c r="N32">
+        <v>0</v>
+      </c>
+      <c r="O32">
+        <v>0</v>
+      </c>
+      <c r="P32">
+        <v>0</v>
+      </c>
+      <c r="Q32">
+        <v>35</v>
+      </c>
+      <c r="R32">
+        <v>27</v>
+      </c>
+      <c r="S32">
+        <v>2</v>
+      </c>
+      <c r="T32">
+        <v>0.46500000000000002</v>
+      </c>
+      <c r="U32">
+        <v>62034200</v>
+      </c>
+      <c r="W32" t="s">
+        <v>33</v>
+      </c>
+      <c r="X32" t="s">
+        <v>34</v>
+      </c>
+      <c r="Y32" t="s">
+        <v>35</v>
+      </c>
+      <c r="Z32" t="s">
+        <v>35</v>
+      </c>
+      <c r="AA32" t="s">
+        <v>35</v>
+      </c>
+    </row>
+    <row r="33" spans="1:27" x14ac:dyDescent="0.3">
+      <c r="A33" t="s">
+        <v>79</v>
+      </c>
+      <c r="B33">
+        <v>32</v>
+      </c>
+      <c r="C33" t="s">
+        <v>75</v>
+      </c>
+      <c r="D33" t="s">
+        <v>29</v>
+      </c>
+      <c r="E33">
+        <v>1499</v>
+      </c>
+      <c r="F33">
+        <v>459</v>
+      </c>
+      <c r="G33">
+        <v>442</v>
+      </c>
+      <c r="H33">
+        <v>1</v>
+      </c>
+      <c r="I33" t="s">
+        <v>30</v>
+      </c>
+      <c r="J33" t="s">
+        <v>31</v>
+      </c>
+      <c r="K33">
+        <v>1</v>
+      </c>
+      <c r="L33">
+        <v>250</v>
+      </c>
+      <c r="M33" t="s">
+        <v>32</v>
+      </c>
+      <c r="N33">
+        <v>0</v>
+      </c>
+      <c r="O33">
+        <v>0</v>
+      </c>
+      <c r="P33">
+        <v>0</v>
+      </c>
+      <c r="Q33">
+        <v>35</v>
+      </c>
+      <c r="R33">
+        <v>27</v>
+      </c>
+      <c r="S33">
+        <v>2</v>
+      </c>
+      <c r="T33">
+        <v>0.46500000000000002</v>
+      </c>
+      <c r="U33">
+        <v>62034200</v>
+      </c>
+      <c r="W33" t="s">
+        <v>33</v>
+      </c>
+      <c r="X33" t="s">
+        <v>34</v>
+      </c>
+      <c r="Y33" t="s">
+        <v>35</v>
+      </c>
+      <c r="Z33" t="s">
+        <v>35</v>
+      </c>
+      <c r="AA33" t="s">
+        <v>35</v>
+      </c>
+    </row>
+    <row r="34" spans="1:27" x14ac:dyDescent="0.3">
+      <c r="A34" t="s">
+        <v>79</v>
+      </c>
+      <c r="B34">
+        <v>30</v>
+      </c>
+      <c r="C34" t="s">
+        <v>76</v>
+      </c>
+      <c r="D34" t="s">
+        <v>29</v>
+      </c>
+      <c r="E34">
+        <v>1499</v>
+      </c>
+      <c r="F34">
+        <v>459</v>
+      </c>
+      <c r="G34">
+        <v>442</v>
+      </c>
+      <c r="H34">
+        <v>1</v>
+      </c>
+      <c r="I34" t="s">
+        <v>30</v>
+      </c>
+      <c r="J34" t="s">
+        <v>31</v>
+      </c>
+      <c r="K34">
+        <v>1</v>
+      </c>
+      <c r="L34">
+        <v>250</v>
+      </c>
+      <c r="M34" t="s">
+        <v>32</v>
+      </c>
+      <c r="N34">
+        <v>0</v>
+      </c>
+      <c r="O34">
+        <v>0</v>
+      </c>
+      <c r="P34">
+        <v>0</v>
+      </c>
+      <c r="Q34">
+        <v>35</v>
+      </c>
+      <c r="R34">
+        <v>27</v>
+      </c>
+      <c r="S34">
+        <v>2</v>
+      </c>
+      <c r="T34">
+        <v>0.46500000000000002</v>
+      </c>
+      <c r="U34">
+        <v>62034200</v>
+      </c>
+      <c r="W34" t="s">
+        <v>33</v>
+      </c>
+      <c r="X34" t="s">
+        <v>34</v>
+      </c>
+      <c r="Y34" t="s">
+        <v>35</v>
+      </c>
+      <c r="Z34" t="s">
+        <v>35</v>
+      </c>
+      <c r="AA34" t="s">
+        <v>35</v>
+      </c>
+    </row>
+    <row r="35" spans="1:27" x14ac:dyDescent="0.3">
+      <c r="A35" t="s">
+        <v>79</v>
+      </c>
+      <c r="B35">
+        <v>28</v>
+      </c>
+      <c r="C35" t="s">
+        <v>77</v>
+      </c>
+      <c r="D35" t="s">
+        <v>29</v>
+      </c>
+      <c r="E35">
+        <v>1499</v>
+      </c>
+      <c r="F35">
+        <v>459</v>
+      </c>
+      <c r="G35">
+        <v>442</v>
+      </c>
+      <c r="H35">
+        <v>1</v>
+      </c>
+      <c r="I35" t="s">
+        <v>30</v>
+      </c>
+      <c r="J35" t="s">
+        <v>31</v>
+      </c>
+      <c r="K35">
+        <v>1</v>
+      </c>
+      <c r="L35">
+        <v>250</v>
+      </c>
+      <c r="M35" t="s">
+        <v>32</v>
+      </c>
+      <c r="N35">
+        <v>0</v>
+      </c>
+      <c r="O35">
+        <v>0</v>
+      </c>
+      <c r="P35">
+        <v>0</v>
+      </c>
+      <c r="Q35">
+        <v>35</v>
+      </c>
+      <c r="R35">
+        <v>27</v>
+      </c>
+      <c r="S35">
+        <v>2</v>
+      </c>
+      <c r="T35">
+        <v>0.46500000000000002</v>
+      </c>
+      <c r="U35">
+        <v>62034200</v>
+      </c>
+      <c r="W35" t="s">
+        <v>33</v>
+      </c>
+      <c r="X35" t="s">
+        <v>34</v>
+      </c>
+      <c r="Y35" t="s">
+        <v>35</v>
+      </c>
+      <c r="Z35" t="s">
+        <v>35</v>
+      </c>
+      <c r="AA35" t="s">
+        <v>35</v>
+      </c>
+    </row>
+    <row r="36" spans="1:27" x14ac:dyDescent="0.3">
+      <c r="A36" t="s">
+        <v>79</v>
+      </c>
+      <c r="B36">
+        <v>26</v>
+      </c>
+      <c r="C36" t="s">
+        <v>78</v>
+      </c>
+      <c r="D36" t="s">
+        <v>29</v>
+      </c>
+      <c r="E36">
+        <v>1499</v>
+      </c>
+      <c r="F36">
+        <v>459</v>
+      </c>
+      <c r="G36">
+        <v>442</v>
+      </c>
+      <c r="H36">
+        <v>1</v>
+      </c>
+      <c r="I36" t="s">
+        <v>30</v>
+      </c>
+      <c r="J36" t="s">
+        <v>31</v>
+      </c>
+      <c r="K36">
+        <v>1</v>
+      </c>
+      <c r="L36">
+        <v>250</v>
+      </c>
+      <c r="M36" t="s">
+        <v>32</v>
+      </c>
+      <c r="N36">
+        <v>0</v>
+      </c>
+      <c r="O36">
+        <v>0</v>
+      </c>
+      <c r="P36">
+        <v>0</v>
+      </c>
+      <c r="Q36">
+        <v>35</v>
+      </c>
+      <c r="R36">
+        <v>27</v>
+      </c>
+      <c r="S36">
+        <v>2</v>
+      </c>
+      <c r="T36">
+        <v>0.46500000000000002</v>
+      </c>
+      <c r="U36">
+        <v>62034200</v>
+      </c>
+      <c r="W36" t="s">
+        <v>33</v>
+      </c>
+      <c r="X36" t="s">
+        <v>34</v>
+      </c>
+      <c r="Y36" t="s">
+        <v>35</v>
+      </c>
+      <c r="Z36" t="s">
+        <v>35</v>
+      </c>
+      <c r="AA36" t="s">
+        <v>35</v>
+      </c>
+    </row>
+    <row r="40" spans="1:27" x14ac:dyDescent="0.3">
       <c r="A40" t="s">
         <v>71</v>
       </c>
     </row>
-    <row r="41" spans="1:1" x14ac:dyDescent="0.25">
+    <row r="41" spans="1:27" x14ac:dyDescent="0.3">
       <c r="A41" t="s">
         <v>72</v>
       </c>
     </row>
-    <row r="42" spans="1:1" x14ac:dyDescent="0.25">
+    <row r="42" spans="1:27" x14ac:dyDescent="0.3">
       <c r="A42" t="s">
         <v>73</v>
       </c>
     </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
-  <pageSetup orientation="portrait" horizontalDpi="4294967295" verticalDpi="4294967295" scale="100" fitToWidth="1" fitToHeight="1"/>
+  <pageSetup orientation="portrait" horizontalDpi="4294967295" verticalDpi="4294967295"/>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
fixed prechecking on queue execution
</commit_message>
<xml_diff>
--- a/Full-LC-AUTO/data inputs/common/Price-Stock-Shipping-inputs.xlsx
+++ b/Full-LC-AUTO/data inputs/common/Price-Stock-Shipping-inputs.xlsx
@@ -1,14 +1,10 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="5" rupBuild="30131"/>
-  <workbookPr filterPrivacy="1"/>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{48F5E4CA-D0C9-4E99-ABF4-C7A03FF330E7}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
-  <bookViews>
-    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="13176" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
-  </bookViews>
+<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" mc:Ignorable="x15">
+  <fileVersion appName="xl" lastEdited="5" lowestEdited="5" rupBuild="9303"/>
+  <workbookPr defaultThemeVersion="164011" filterPrivacy="1"/>
   <sheets>
-    <sheet name="Product Inputs" sheetId="1" r:id="rId1"/>
+    <sheet sheetId="1" name="Product Inputs" state="visible" r:id="rId4"/>
   </sheets>
   <calcPr calcId="171027"/>
 </workbook>
@@ -230,6 +226,24 @@
     <t>FB-S-TRACK-PANT-BLACk-01-</t>
   </si>
   <si>
+    <t>White-Baggy</t>
+  </si>
+  <si>
+    <t>FB-34-WHITE-Baggy-Plain-Jeans-BEPJ-</t>
+  </si>
+  <si>
+    <t>FB-32-WHITE-Baggy-Plain-Jeans-BEPJ-</t>
+  </si>
+  <si>
+    <t>FB-30-WHITE-Baggy-Plain-Jeans-BEPJ-</t>
+  </si>
+  <si>
+    <t>FB-28-WHITE-Baggy-Plain-Jeans-BEPJ-</t>
+  </si>
+  <si>
+    <t>FB-26-WHITE-Baggy-Plain-Jeans-BEPJ-</t>
+  </si>
+  <si>
     <t>Use one row per product/size combination.</t>
   </si>
   <si>
@@ -237,37 +251,19 @@
   </si>
   <si>
     <t>Do not rename headers.</t>
-  </si>
-  <si>
-    <t>FB-34-WHITE-Baggy-Plain-Jeans-BEPJ-</t>
-  </si>
-  <si>
-    <t>FB-32-WHITE-Baggy-Plain-Jeans-BEPJ-</t>
-  </si>
-  <si>
-    <t>FB-30-WHITE-Baggy-Plain-Jeans-BEPJ-</t>
-  </si>
-  <si>
-    <t>FB-28-WHITE-Baggy-Plain-Jeans-BEPJ-</t>
-  </si>
-  <si>
-    <t>FB-26-WHITE-Baggy-Plain-Jeans-BEPJ-</t>
-  </si>
-  <si>
-    <t>White-Baggy</t>
   </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
-<styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
+<styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" mc:Ignorable="x14ac x16r2">
   <fonts count="1" x14ac:knownFonts="1">
     <font>
-      <sz val="11"/>
       <color theme="1"/>
-      <name val="Calibri"/>
       <family val="2"/>
       <scheme val="minor"/>
+      <sz val="11"/>
+      <name val="Calibri"/>
     </font>
   </fonts>
   <fills count="2">
@@ -630,30 +626,30 @@
 </file>
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
   <dimension ref="A1:AA42"/>
-  <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
+  <sheetFormatPr defaultRowHeight="15" outlineLevelRow="0" outlineLevelCol="0" x14ac:dyDescent="55"/>
   <cols>
-    <col min="1" max="1" width="42.109375" customWidth="1"/>
-    <col min="2" max="2" width="26.5546875" customWidth="1"/>
-    <col min="3" max="3" width="35.88671875" customWidth="1"/>
-    <col min="4" max="4" width="37.6640625" customWidth="1"/>
-    <col min="5" max="6" width="30.109375" customWidth="1"/>
-    <col min="7" max="8" width="42.109375" customWidth="1"/>
-    <col min="9" max="9" width="37.6640625" customWidth="1"/>
-    <col min="10" max="10" width="41.109375" customWidth="1"/>
-    <col min="11" max="11" width="39.5546875" customWidth="1"/>
-    <col min="12" max="12" width="30.109375" customWidth="1"/>
-    <col min="13" max="16" width="42.109375" customWidth="1"/>
-    <col min="17" max="21" width="30.109375" customWidth="1"/>
-    <col min="22" max="22" width="31.88671875" customWidth="1"/>
-    <col min="23" max="23" width="30.109375" customWidth="1"/>
-    <col min="24" max="25" width="42.109375" customWidth="1"/>
-    <col min="26" max="26" width="37.6640625" customWidth="1"/>
-    <col min="27" max="27" width="41.109375" customWidth="1"/>
+    <col min="1" max="1" width="42.142857142857146" customWidth="1"/>
+    <col min="2" max="2" width="26.571428571428573" customWidth="1"/>
+    <col min="3" max="3" width="35.857142857142854" customWidth="1"/>
+    <col min="4" max="4" width="37.714285714285715" customWidth="1"/>
+    <col min="5" max="6" width="30.142857142857142" customWidth="1"/>
+    <col min="7" max="8" width="42.142857142857146" customWidth="1"/>
+    <col min="9" max="9" width="37.714285714285715" customWidth="1"/>
+    <col min="10" max="10" width="41.142857142857146" customWidth="1"/>
+    <col min="11" max="11" width="39.57142857142857" customWidth="1"/>
+    <col min="12" max="12" width="30.142857142857142" customWidth="1"/>
+    <col min="13" max="16" width="42.142857142857146" customWidth="1"/>
+    <col min="17" max="21" width="30.142857142857142" customWidth="1"/>
+    <col min="22" max="22" width="31.857142857142858" customWidth="1"/>
+    <col min="23" max="23" width="30.142857142857142" customWidth="1"/>
+    <col min="24" max="25" width="42.142857142857146" customWidth="1"/>
+    <col min="26" max="26" width="37.714285714285715" customWidth="1"/>
+    <col min="27" max="27" width="41.142857142857146" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:27" x14ac:dyDescent="0.3">
+    <row r="1" spans="1:27" x14ac:dyDescent="0.25">
       <c r="A1" t="s">
         <v>0</v>
       </c>
@@ -736,7 +732,7 @@
         <v>26</v>
       </c>
     </row>
-    <row r="2" spans="1:27" x14ac:dyDescent="0.3">
+    <row r="2" spans="1:27" x14ac:dyDescent="0.25">
       <c r="A2" t="s">
         <v>27</v>
       </c>
@@ -795,7 +791,7 @@
         <v>2</v>
       </c>
       <c r="T2">
-        <v>0.46500000000000002</v>
+        <v>0.465</v>
       </c>
       <c r="U2">
         <v>62034200</v>
@@ -816,7 +812,7 @@
         <v>35</v>
       </c>
     </row>
-    <row r="3" spans="1:27" x14ac:dyDescent="0.3">
+    <row r="3" spans="1:27" x14ac:dyDescent="0.25">
       <c r="A3" t="s">
         <v>27</v>
       </c>
@@ -875,7 +871,7 @@
         <v>2</v>
       </c>
       <c r="T3">
-        <v>0.46500000000000002</v>
+        <v>0.465</v>
       </c>
       <c r="U3">
         <v>62034200</v>
@@ -896,7 +892,7 @@
         <v>35</v>
       </c>
     </row>
-    <row r="4" spans="1:27" x14ac:dyDescent="0.3">
+    <row r="4" spans="1:27" x14ac:dyDescent="0.25">
       <c r="A4" t="s">
         <v>27</v>
       </c>
@@ -955,7 +951,7 @@
         <v>2</v>
       </c>
       <c r="T4">
-        <v>0.46500000000000002</v>
+        <v>0.465</v>
       </c>
       <c r="U4">
         <v>62034200</v>
@@ -976,7 +972,7 @@
         <v>35</v>
       </c>
     </row>
-    <row r="5" spans="1:27" x14ac:dyDescent="0.3">
+    <row r="5" spans="1:27" x14ac:dyDescent="0.25">
       <c r="A5" t="s">
         <v>27</v>
       </c>
@@ -1035,7 +1031,7 @@
         <v>2</v>
       </c>
       <c r="T5">
-        <v>0.46500000000000002</v>
+        <v>0.465</v>
       </c>
       <c r="U5">
         <v>62034200</v>
@@ -1056,7 +1052,7 @@
         <v>35</v>
       </c>
     </row>
-    <row r="6" spans="1:27" x14ac:dyDescent="0.3">
+    <row r="6" spans="1:27" x14ac:dyDescent="0.25">
       <c r="A6" t="s">
         <v>27</v>
       </c>
@@ -1115,7 +1111,7 @@
         <v>2</v>
       </c>
       <c r="T6">
-        <v>0.46500000000000002</v>
+        <v>0.465</v>
       </c>
       <c r="U6">
         <v>62034200</v>
@@ -1136,7 +1132,7 @@
         <v>35</v>
       </c>
     </row>
-    <row r="7" spans="1:27" x14ac:dyDescent="0.3">
+    <row r="7" spans="1:27" x14ac:dyDescent="0.25">
       <c r="A7" t="s">
         <v>40</v>
       </c>
@@ -1195,7 +1191,7 @@
         <v>2</v>
       </c>
       <c r="T7">
-        <v>0.46500000000000002</v>
+        <v>0.465</v>
       </c>
       <c r="U7">
         <v>62034200</v>
@@ -1216,7 +1212,7 @@
         <v>35</v>
       </c>
     </row>
-    <row r="8" spans="1:27" x14ac:dyDescent="0.3">
+    <row r="8" spans="1:27" x14ac:dyDescent="0.25">
       <c r="A8" t="s">
         <v>40</v>
       </c>
@@ -1275,7 +1271,7 @@
         <v>2</v>
       </c>
       <c r="T8">
-        <v>0.46500000000000002</v>
+        <v>0.465</v>
       </c>
       <c r="U8">
         <v>62034200</v>
@@ -1296,7 +1292,7 @@
         <v>35</v>
       </c>
     </row>
-    <row r="9" spans="1:27" x14ac:dyDescent="0.3">
+    <row r="9" spans="1:27" x14ac:dyDescent="0.25">
       <c r="A9" t="s">
         <v>40</v>
       </c>
@@ -1355,7 +1351,7 @@
         <v>2</v>
       </c>
       <c r="T9">
-        <v>0.46500000000000002</v>
+        <v>0.465</v>
       </c>
       <c r="U9">
         <v>62034200</v>
@@ -1376,7 +1372,7 @@
         <v>35</v>
       </c>
     </row>
-    <row r="10" spans="1:27" x14ac:dyDescent="0.3">
+    <row r="10" spans="1:27" x14ac:dyDescent="0.25">
       <c r="A10" t="s">
         <v>40</v>
       </c>
@@ -1435,7 +1431,7 @@
         <v>2</v>
       </c>
       <c r="T10">
-        <v>0.46500000000000002</v>
+        <v>0.465</v>
       </c>
       <c r="U10">
         <v>62034200</v>
@@ -1456,7 +1452,7 @@
         <v>35</v>
       </c>
     </row>
-    <row r="11" spans="1:27" x14ac:dyDescent="0.3">
+    <row r="11" spans="1:27" x14ac:dyDescent="0.25">
       <c r="A11" t="s">
         <v>40</v>
       </c>
@@ -1515,7 +1511,7 @@
         <v>2</v>
       </c>
       <c r="T11">
-        <v>0.46500000000000002</v>
+        <v>0.465</v>
       </c>
       <c r="U11">
         <v>62034200</v>
@@ -1536,7 +1532,7 @@
         <v>35</v>
       </c>
     </row>
-    <row r="12" spans="1:27" x14ac:dyDescent="0.3">
+    <row r="12" spans="1:27" x14ac:dyDescent="0.25">
       <c r="A12" t="s">
         <v>47</v>
       </c>
@@ -1616,7 +1612,7 @@
         <v>35</v>
       </c>
     </row>
-    <row r="13" spans="1:27" x14ac:dyDescent="0.3">
+    <row r="13" spans="1:27" x14ac:dyDescent="0.25">
       <c r="A13" t="s">
         <v>47</v>
       </c>
@@ -1696,7 +1692,7 @@
         <v>35</v>
       </c>
     </row>
-    <row r="14" spans="1:27" x14ac:dyDescent="0.3">
+    <row r="14" spans="1:27" x14ac:dyDescent="0.25">
       <c r="A14" t="s">
         <v>47</v>
       </c>
@@ -1776,7 +1772,7 @@
         <v>35</v>
       </c>
     </row>
-    <row r="15" spans="1:27" x14ac:dyDescent="0.3">
+    <row r="15" spans="1:27" x14ac:dyDescent="0.25">
       <c r="A15" t="s">
         <v>54</v>
       </c>
@@ -1856,7 +1852,7 @@
         <v>35</v>
       </c>
     </row>
-    <row r="16" spans="1:27" x14ac:dyDescent="0.3">
+    <row r="16" spans="1:27" x14ac:dyDescent="0.25">
       <c r="A16" t="s">
         <v>54</v>
       </c>
@@ -1936,7 +1932,7 @@
         <v>35</v>
       </c>
     </row>
-    <row r="17" spans="1:27" x14ac:dyDescent="0.3">
+    <row r="17" spans="1:27" x14ac:dyDescent="0.25">
       <c r="A17" t="s">
         <v>54</v>
       </c>
@@ -2016,7 +2012,7 @@
         <v>35</v>
       </c>
     </row>
-    <row r="18" spans="1:27" x14ac:dyDescent="0.3">
+    <row r="18" spans="1:27" x14ac:dyDescent="0.25">
       <c r="A18" t="s">
         <v>54</v>
       </c>
@@ -2096,7 +2092,7 @@
         <v>35</v>
       </c>
     </row>
-    <row r="19" spans="1:27" x14ac:dyDescent="0.3">
+    <row r="19" spans="1:27" x14ac:dyDescent="0.25">
       <c r="A19" t="s">
         <v>54</v>
       </c>
@@ -2176,7 +2172,7 @@
         <v>35</v>
       </c>
     </row>
-    <row r="20" spans="1:27" x14ac:dyDescent="0.3">
+    <row r="20" spans="1:27" x14ac:dyDescent="0.25">
       <c r="A20" t="s">
         <v>54</v>
       </c>
@@ -2256,7 +2252,7 @@
         <v>35</v>
       </c>
     </row>
-    <row r="21" spans="1:27" x14ac:dyDescent="0.3">
+    <row r="21" spans="1:27" x14ac:dyDescent="0.25">
       <c r="A21" t="s">
         <v>54</v>
       </c>
@@ -2336,7 +2332,7 @@
         <v>35</v>
       </c>
     </row>
-    <row r="22" spans="1:27" x14ac:dyDescent="0.3">
+    <row r="22" spans="1:27" x14ac:dyDescent="0.25">
       <c r="A22" t="s">
         <v>54</v>
       </c>
@@ -2416,7 +2412,7 @@
         <v>35</v>
       </c>
     </row>
-    <row r="23" spans="1:27" x14ac:dyDescent="0.3">
+    <row r="23" spans="1:27" x14ac:dyDescent="0.25">
       <c r="A23" t="s">
         <v>60</v>
       </c>
@@ -2475,7 +2471,7 @@
         <v>2</v>
       </c>
       <c r="T23">
-        <v>0.46500000000000002</v>
+        <v>0.465</v>
       </c>
       <c r="U23">
         <v>62034200</v>
@@ -2496,7 +2492,7 @@
         <v>35</v>
       </c>
     </row>
-    <row r="24" spans="1:27" x14ac:dyDescent="0.3">
+    <row r="24" spans="1:27" x14ac:dyDescent="0.25">
       <c r="A24" t="s">
         <v>60</v>
       </c>
@@ -2555,7 +2551,7 @@
         <v>2</v>
       </c>
       <c r="T24">
-        <v>0.46500000000000002</v>
+        <v>0.465</v>
       </c>
       <c r="U24">
         <v>62034200</v>
@@ -2576,7 +2572,7 @@
         <v>35</v>
       </c>
     </row>
-    <row r="25" spans="1:27" x14ac:dyDescent="0.3">
+    <row r="25" spans="1:27" x14ac:dyDescent="0.25">
       <c r="A25" t="s">
         <v>60</v>
       </c>
@@ -2635,7 +2631,7 @@
         <v>2</v>
       </c>
       <c r="T25">
-        <v>0.46500000000000002</v>
+        <v>0.465</v>
       </c>
       <c r="U25">
         <v>62034200</v>
@@ -2656,7 +2652,7 @@
         <v>35</v>
       </c>
     </row>
-    <row r="26" spans="1:27" x14ac:dyDescent="0.3">
+    <row r="26" spans="1:27" x14ac:dyDescent="0.25">
       <c r="A26" t="s">
         <v>60</v>
       </c>
@@ -2715,7 +2711,7 @@
         <v>2</v>
       </c>
       <c r="T26">
-        <v>0.46500000000000002</v>
+        <v>0.465</v>
       </c>
       <c r="U26">
         <v>62034200</v>
@@ -2736,7 +2732,7 @@
         <v>35</v>
       </c>
     </row>
-    <row r="27" spans="1:27" x14ac:dyDescent="0.3">
+    <row r="27" spans="1:27" x14ac:dyDescent="0.25">
       <c r="A27" t="s">
         <v>60</v>
       </c>
@@ -2795,7 +2791,7 @@
         <v>2</v>
       </c>
       <c r="T27">
-        <v>0.46500000000000002</v>
+        <v>0.465</v>
       </c>
       <c r="U27">
         <v>62034200</v>
@@ -2816,7 +2812,7 @@
         <v>35</v>
       </c>
     </row>
-    <row r="28" spans="1:27" x14ac:dyDescent="0.3">
+    <row r="28" spans="1:27" x14ac:dyDescent="0.25">
       <c r="A28" t="s">
         <v>66</v>
       </c>
@@ -2896,7 +2892,7 @@
         <v>35</v>
       </c>
     </row>
-    <row r="29" spans="1:27" x14ac:dyDescent="0.3">
+    <row r="29" spans="1:27" x14ac:dyDescent="0.25">
       <c r="A29" t="s">
         <v>66</v>
       </c>
@@ -2976,7 +2972,7 @@
         <v>35</v>
       </c>
     </row>
-    <row r="30" spans="1:27" x14ac:dyDescent="0.3">
+    <row r="30" spans="1:27" x14ac:dyDescent="0.25">
       <c r="A30" t="s">
         <v>66</v>
       </c>
@@ -3056,7 +3052,7 @@
         <v>35</v>
       </c>
     </row>
-    <row r="31" spans="1:27" x14ac:dyDescent="0.3">
+    <row r="31" spans="1:27" x14ac:dyDescent="0.25">
       <c r="A31" t="s">
         <v>66</v>
       </c>
@@ -3136,27 +3132,27 @@
         <v>35</v>
       </c>
     </row>
-    <row r="32" spans="1:27" x14ac:dyDescent="0.3">
+    <row r="32" spans="1:27" x14ac:dyDescent="0.25">
       <c r="A32" t="s">
-        <v>79</v>
+        <v>71</v>
       </c>
       <c r="B32">
         <v>34</v>
       </c>
       <c r="C32" t="s">
-        <v>74</v>
+        <v>72</v>
       </c>
       <c r="D32" t="s">
-        <v>29</v>
+        <v>46</v>
       </c>
       <c r="E32">
         <v>1499</v>
       </c>
       <c r="F32">
-        <v>459</v>
+        <v>429</v>
       </c>
       <c r="G32">
-        <v>442</v>
+        <v>429</v>
       </c>
       <c r="H32">
         <v>1</v>
@@ -3195,7 +3191,7 @@
         <v>2</v>
       </c>
       <c r="T32">
-        <v>0.46500000000000002</v>
+        <v>0.465</v>
       </c>
       <c r="U32">
         <v>62034200</v>
@@ -3216,15 +3212,15 @@
         <v>35</v>
       </c>
     </row>
-    <row r="33" spans="1:27" x14ac:dyDescent="0.3">
+    <row r="33" spans="1:27" x14ac:dyDescent="0.25">
       <c r="A33" t="s">
-        <v>79</v>
+        <v>71</v>
       </c>
       <c r="B33">
         <v>32</v>
       </c>
       <c r="C33" t="s">
-        <v>75</v>
+        <v>73</v>
       </c>
       <c r="D33" t="s">
         <v>29</v>
@@ -3233,10 +3229,10 @@
         <v>1499</v>
       </c>
       <c r="F33">
-        <v>459</v>
+        <v>419</v>
       </c>
       <c r="G33">
-        <v>442</v>
+        <v>419</v>
       </c>
       <c r="H33">
         <v>1</v>
@@ -3275,7 +3271,7 @@
         <v>2</v>
       </c>
       <c r="T33">
-        <v>0.46500000000000002</v>
+        <v>0.465</v>
       </c>
       <c r="U33">
         <v>62034200</v>
@@ -3296,15 +3292,15 @@
         <v>35</v>
       </c>
     </row>
-    <row r="34" spans="1:27" x14ac:dyDescent="0.3">
+    <row r="34" spans="1:27" x14ac:dyDescent="0.25">
       <c r="A34" t="s">
-        <v>79</v>
+        <v>71</v>
       </c>
       <c r="B34">
         <v>30</v>
       </c>
       <c r="C34" t="s">
-        <v>76</v>
+        <v>74</v>
       </c>
       <c r="D34" t="s">
         <v>29</v>
@@ -3313,10 +3309,10 @@
         <v>1499</v>
       </c>
       <c r="F34">
-        <v>459</v>
+        <v>419</v>
       </c>
       <c r="G34">
-        <v>442</v>
+        <v>419</v>
       </c>
       <c r="H34">
         <v>1</v>
@@ -3355,7 +3351,7 @@
         <v>2</v>
       </c>
       <c r="T34">
-        <v>0.46500000000000002</v>
+        <v>0.465</v>
       </c>
       <c r="U34">
         <v>62034200</v>
@@ -3376,15 +3372,15 @@
         <v>35</v>
       </c>
     </row>
-    <row r="35" spans="1:27" x14ac:dyDescent="0.3">
+    <row r="35" spans="1:27" x14ac:dyDescent="0.25">
       <c r="A35" t="s">
-        <v>79</v>
+        <v>71</v>
       </c>
       <c r="B35">
         <v>28</v>
       </c>
       <c r="C35" t="s">
-        <v>77</v>
+        <v>75</v>
       </c>
       <c r="D35" t="s">
         <v>29</v>
@@ -3393,10 +3389,10 @@
         <v>1499</v>
       </c>
       <c r="F35">
-        <v>459</v>
+        <v>419</v>
       </c>
       <c r="G35">
-        <v>442</v>
+        <v>419</v>
       </c>
       <c r="H35">
         <v>1</v>
@@ -3435,7 +3431,7 @@
         <v>2</v>
       </c>
       <c r="T35">
-        <v>0.46500000000000002</v>
+        <v>0.465</v>
       </c>
       <c r="U35">
         <v>62034200</v>
@@ -3456,27 +3452,27 @@
         <v>35</v>
       </c>
     </row>
-    <row r="36" spans="1:27" x14ac:dyDescent="0.3">
+    <row r="36" spans="1:27" x14ac:dyDescent="0.25">
       <c r="A36" t="s">
-        <v>79</v>
+        <v>71</v>
       </c>
       <c r="B36">
         <v>26</v>
       </c>
       <c r="C36" t="s">
-        <v>78</v>
+        <v>76</v>
       </c>
       <c r="D36" t="s">
-        <v>29</v>
+        <v>46</v>
       </c>
       <c r="E36">
         <v>1499</v>
       </c>
       <c r="F36">
-        <v>459</v>
+        <v>419</v>
       </c>
       <c r="G36">
-        <v>442</v>
+        <v>419</v>
       </c>
       <c r="H36">
         <v>1</v>
@@ -3515,7 +3511,7 @@
         <v>2</v>
       </c>
       <c r="T36">
-        <v>0.46500000000000002</v>
+        <v>0.465</v>
       </c>
       <c r="U36">
         <v>62034200</v>
@@ -3536,23 +3532,24 @@
         <v>35</v>
       </c>
     </row>
-    <row r="40" spans="1:27" x14ac:dyDescent="0.3">
+    <row r="37" spans="7:7" x14ac:dyDescent="0.25"/>
+    <row r="40" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A40" t="s">
-        <v>71</v>
-      </c>
-    </row>
-    <row r="41" spans="1:27" x14ac:dyDescent="0.3">
+        <v>77</v>
+      </c>
+    </row>
+    <row r="41" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A41" t="s">
-        <v>72</v>
-      </c>
-    </row>
-    <row r="42" spans="1:27" x14ac:dyDescent="0.3">
+        <v>78</v>
+      </c>
+    </row>
+    <row r="42" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A42" t="s">
-        <v>73</v>
+        <v>79</v>
       </c>
     </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
-  <pageSetup orientation="portrait" horizontalDpi="4294967295" verticalDpi="4294967295"/>
+  <pageSetup orientation="portrait" horizontalDpi="4294967295" verticalDpi="4294967295" scale="100" fitToWidth="1" fitToHeight="1"/>
 </worksheet>
 </file>
</xml_diff>